<commit_message>
[CBDDO & ZT-OT] Fix Framework URNs
</commit_message>
<xml_diff>
--- a/tools/excel/CBDDO/CBDDO-BIGR.xlsx
+++ b/tools/excel/CBDDO/CBDDO-BIGR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\excel\CBDDO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC77181-67FD-44FF-89A1-F3FC33490B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE546B0-3848-4C0D-9129-F7DB2EF62C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-8660" windowWidth="38620" windowHeight="21820" tabRatio="907" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="907" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -10056,16 +10056,16 @@
 Anlık görüntüler şifreli olarak korunmakta mıdır?</t>
   </si>
   <si>
-    <t>urn:intuitem:risk:library:CBDDO_BIGR</t>
-  </si>
-  <si>
-    <t>urn:intuitem:risk:req_node:CBDDO_BIGR</t>
-  </si>
-  <si>
-    <t>urn:intuitem:risk:framework:CBDDO_BIGR</t>
-  </si>
-  <si>
     <t>CBDDO_BIGR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">urn:intuitem:risk:req_node:cbddo_bigr </t>
+  </si>
+  <si>
+    <t>urn:intuitem:risk:framework:cbddo_bigr</t>
+  </si>
+  <si>
+    <t>urn:intuitem:risk:library:cbddo_bigr</t>
   </si>
 </sst>
 </file>
@@ -11371,7 +11371,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>2897</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -11395,7 +11395,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>2900</v>
+        <v>2897</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -11493,7 +11493,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>2900</v>
+        <v>2897</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -12513,7 +12513,7 @@
       <c r="J33" s="40"/>
       <c r="K33" s="43"/>
     </row>
-    <row r="34" spans="1:11" s="19" customFormat="1" ht="97.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" s="19" customFormat="1" ht="111" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="41" t="s">
         <v>21</v>
       </c>
@@ -13334,7 +13334,7 @@
       <c r="J62" s="40"/>
       <c r="K62" s="43"/>
     </row>
-    <row r="63" spans="1:11" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="41" t="s">
         <v>21</v>
       </c>
@@ -14986,7 +14986,7 @@
         <v>2521</v>
       </c>
     </row>
-    <row r="121" spans="1:11" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A121" s="41" t="s">
         <v>21</v>
       </c>
@@ -16319,7 +16319,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="168" spans="1:11" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:11" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A168" s="41" t="s">
         <v>21</v>
       </c>
@@ -17198,7 +17198,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="199" spans="1:11" ht="111" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:11" ht="124.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A199" s="41" t="s">
         <v>21</v>
       </c>
@@ -17401,7 +17401,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="206" spans="1:11" ht="193.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:11" ht="207.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A206" s="41" t="s">
         <v>21</v>
       </c>
@@ -18096,7 +18096,7 @@
         <v>2512</v>
       </c>
     </row>
-    <row r="231" spans="1:11" ht="180" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:11" ht="193.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A231" s="41" t="s">
         <v>21</v>
       </c>
@@ -18511,7 +18511,7 @@
         <v>2655</v>
       </c>
     </row>
-    <row r="246" spans="1:11" ht="111" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:11" ht="124.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A246" s="41" t="s">
         <v>21</v>
       </c>
@@ -24361,7 +24361,7 @@
         <v>2514</v>
       </c>
     </row>
-    <row r="456" spans="1:11" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="456" spans="1:11" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A456" s="41" t="s">
         <v>21</v>
       </c>
@@ -26531,7 +26531,7 @@
       <c r="J535" s="47"/>
       <c r="K535" s="43"/>
     </row>
-    <row r="536" spans="1:11" ht="138.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:11" ht="152.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A536" s="41" t="s">
         <v>21</v>
       </c>
@@ -28086,7 +28086,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="591" spans="1:11" ht="97.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="591" spans="1:11" ht="111" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A591" s="41" t="s">
         <v>21</v>
       </c>
@@ -29939,7 +29939,7 @@
         <v>2518</v>
       </c>
     </row>
-    <row r="658" spans="1:11" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="658" spans="1:11" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A658" s="41" t="s">
         <v>21</v>
       </c>
@@ -30827,7 +30827,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="690" spans="1:11" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="690" spans="1:11" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A690" s="41" t="s">
         <v>21</v>
       </c>
@@ -31059,7 +31059,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="698" spans="1:11" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="698" spans="1:11" ht="97.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A698" s="41" t="s">
         <v>21</v>
       </c>

</xml_diff>